<commit_message>
Refresh OpenAI extraction cache and regenerate Beacon outputs.
Re-ran the full --refresh-cache pipeline: 31 native-text and 4 vision extractions, no local fallback, all workbooks and audit files regenerated.

Co-authored-by: anthonyleedu <anthonyleedu@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/lisa_reconciliation.xlsx
+++ b/output/lisa_reconciliation.xlsx
@@ -849,136 +849,136 @@
     <t>gpt-4o-mini</t>
   </si>
   <si>
+    <t>d41e5965ac0d</t>
+  </si>
+  <si>
+    <t>UNKNOWN</t>
+  </si>
+  <si>
+    <t>1e36a3bb8230</t>
+  </si>
+  <si>
+    <t>b109ebc6b485</t>
+  </si>
+  <si>
+    <t>527671baf80d</t>
+  </si>
+  <si>
+    <t>78e12caee3d0</t>
+  </si>
+  <si>
+    <t>3a93a05eccfb</t>
+  </si>
+  <si>
+    <t>498d9e57c248</t>
+  </si>
+  <si>
+    <t>666ddb95cb5e</t>
+  </si>
+  <si>
+    <t>171acbfe62b4</t>
+  </si>
+  <si>
+    <t>CONTINENTAL QUALITY HEAT TREAT</t>
+  </si>
+  <si>
+    <t>VISION</t>
+  </si>
+  <si>
+    <t>bccc160e1d7a</t>
+  </si>
+  <si>
+    <t>ce09a43a057d</t>
+  </si>
+  <si>
+    <t>0335b5f9c32c</t>
+  </si>
+  <si>
+    <t>955c6553efee</t>
+  </si>
+  <si>
+    <t>803cca7204dd</t>
+  </si>
+  <si>
+    <t>5c96fdc23f2b</t>
+  </si>
+  <si>
+    <t>da7824243c72</t>
+  </si>
+  <si>
+    <t>0f0f0358478e</t>
+  </si>
+  <si>
+    <t>33d82e21944f</t>
+  </si>
+  <si>
+    <t>22e8e11993b9</t>
+  </si>
+  <si>
+    <t>c4b891a575c5</t>
+  </si>
+  <si>
+    <t>LIB-PO-9240</t>
+  </si>
+  <si>
+    <t>liberty_02.pdf</t>
+  </si>
+  <si>
+    <t>064f140583b6</t>
+  </si>
+  <si>
+    <t>df73e325ff79</t>
+  </si>
+  <si>
+    <t>RECEIPT_ONLY</t>
+  </si>
+  <si>
+    <t>RECEIPT_ACKNOWLEDGED_NO_SCHEDULE</t>
+  </si>
+  <si>
+    <t>e091bfef23ea</t>
+  </si>
+  <si>
+    <t>CAD</t>
+  </si>
+  <si>
+    <t>e8a55dd92b82</t>
+  </si>
+  <si>
+    <t>57987fd5631a</t>
+  </si>
+  <si>
+    <t>cb089f26bc54</t>
+  </si>
+  <si>
+    <t>7824420c3184</t>
+  </si>
+  <si>
+    <t>7dbe09998647</t>
+  </si>
+  <si>
+    <t>9e089392ebf2</t>
+  </si>
+  <si>
+    <t>af20c417f7de</t>
+  </si>
+  <si>
+    <t>quickship_01.pdf</t>
+  </si>
+  <si>
+    <t>450c226ef559</t>
+  </si>
+  <si>
+    <t>SUPERSEDED</t>
+  </si>
+  <si>
+    <t>8c7d47657ef5</t>
+  </si>
+  <si>
+    <t>REVISION</t>
+  </si>
+  <si>
     <t>Y</t>
-  </si>
-  <si>
-    <t>d41e5965ac0d</t>
-  </si>
-  <si>
-    <t>1e36a3bb8230</t>
-  </si>
-  <si>
-    <t>b109ebc6b485</t>
-  </si>
-  <si>
-    <t>527671baf80d</t>
-  </si>
-  <si>
-    <t>78e12caee3d0</t>
-  </si>
-  <si>
-    <t>3a93a05eccfb</t>
-  </si>
-  <si>
-    <t>498d9e57c248</t>
-  </si>
-  <si>
-    <t>666ddb95cb5e</t>
-  </si>
-  <si>
-    <t>171acbfe62b4</t>
-  </si>
-  <si>
-    <t>CONTINENTAL QUALITY HEAT TREAT</t>
-  </si>
-  <si>
-    <t>UNKNOWN</t>
-  </si>
-  <si>
-    <t>VISION</t>
-  </si>
-  <si>
-    <t>bccc160e1d7a</t>
-  </si>
-  <si>
-    <t>ce09a43a057d</t>
-  </si>
-  <si>
-    <t>0335b5f9c32c</t>
-  </si>
-  <si>
-    <t>955c6553efee</t>
-  </si>
-  <si>
-    <t>803cca7204dd</t>
-  </si>
-  <si>
-    <t>5c96fdc23f2b</t>
-  </si>
-  <si>
-    <t>da7824243c72</t>
-  </si>
-  <si>
-    <t>0f0f0358478e</t>
-  </si>
-  <si>
-    <t>33d82e21944f</t>
-  </si>
-  <si>
-    <t>22e8e11993b9</t>
-  </si>
-  <si>
-    <t>c4b891a575c5</t>
-  </si>
-  <si>
-    <t>LIB-PO-9240</t>
-  </si>
-  <si>
-    <t>liberty_02.pdf</t>
-  </si>
-  <si>
-    <t>064f140583b6</t>
-  </si>
-  <si>
-    <t>df73e325ff79</t>
-  </si>
-  <si>
-    <t>RECEIPT_ONLY</t>
-  </si>
-  <si>
-    <t>RECEIPT_ACKNOWLEDGED_NO_SCHEDULE</t>
-  </si>
-  <si>
-    <t>e091bfef23ea</t>
-  </si>
-  <si>
-    <t>CAD</t>
-  </si>
-  <si>
-    <t>e8a55dd92b82</t>
-  </si>
-  <si>
-    <t>57987fd5631a</t>
-  </si>
-  <si>
-    <t>cb089f26bc54</t>
-  </si>
-  <si>
-    <t>7824420c3184</t>
-  </si>
-  <si>
-    <t>7dbe09998647</t>
-  </si>
-  <si>
-    <t>9e089392ebf2</t>
-  </si>
-  <si>
-    <t>af20c417f7de</t>
-  </si>
-  <si>
-    <t>quickship_01.pdf</t>
-  </si>
-  <si>
-    <t>450c226ef559</t>
-  </si>
-  <si>
-    <t>SUPERSEDED</t>
-  </si>
-  <si>
-    <t>8c7d47657ef5</t>
-  </si>
-  <si>
-    <t>REVISION</t>
   </si>
   <si>
     <t>e614ec5ee714</t>
@@ -8276,7 +8276,7 @@
         <v>272</v>
       </c>
       <c r="R2" s="16" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="S2" s="16"/>
       <c r="T2" s="16"/>
@@ -8286,7 +8286,7 @@
         <v>44</v>
       </c>
       <c r="B3" s="16" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C3" s="16" t="s">
         <v>67</v>
@@ -8304,7 +8304,7 @@
         <v>268</v>
       </c>
       <c r="H3" s="16" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
       <c r="I3" s="16" t="s">
         <v>46</v>
@@ -8330,7 +8330,7 @@
         <v>272</v>
       </c>
       <c r="R3" s="16" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="S3" s="16"/>
       <c r="T3" s="16"/>
@@ -8384,7 +8384,7 @@
         <v>272</v>
       </c>
       <c r="R4" s="16" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="S4" s="16"/>
       <c r="T4" s="16"/>
@@ -8438,7 +8438,7 @@
         <v>272</v>
       </c>
       <c r="R5" s="16" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="S5" s="16"/>
       <c r="T5" s="16"/>
@@ -8492,7 +8492,7 @@
         <v>272</v>
       </c>
       <c r="R6" s="16" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="S6" s="16"/>
       <c r="T6" s="16"/>
@@ -8546,7 +8546,7 @@
         <v>272</v>
       </c>
       <c r="R7" s="16" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="S7" s="16"/>
       <c r="T7" s="16"/>
@@ -8600,7 +8600,7 @@
         <v>272</v>
       </c>
       <c r="R8" s="16" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="S8" s="16"/>
       <c r="T8" s="16"/>
@@ -8654,7 +8654,7 @@
         <v>272</v>
       </c>
       <c r="R9" s="16" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="S9" s="16"/>
       <c r="T9" s="16"/>
@@ -8708,7 +8708,7 @@
         <v>272</v>
       </c>
       <c r="R10" s="16" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="S10" s="16"/>
       <c r="T10" s="16"/>
@@ -8734,7 +8734,7 @@
         <v>268</v>
       </c>
       <c r="H11" s="16" t="s">
-        <v>284</v>
+        <v>274</v>
       </c>
       <c r="I11" s="16" t="s">
         <v>46</v>
@@ -8752,13 +8752,13 @@
         <v>1</v>
       </c>
       <c r="P11" s="16" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="Q11" s="16" t="s">
         <v>272</v>
       </c>
       <c r="R11" s="16" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="S11" s="16"/>
       <c r="T11" s="16"/>
@@ -8768,7 +8768,7 @@
         <v>182</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="C12" s="16" t="s">
         <v>283</v>
@@ -8784,7 +8784,7 @@
         <v>268</v>
       </c>
       <c r="H12" s="16" t="s">
-        <v>284</v>
+        <v>274</v>
       </c>
       <c r="I12" s="16" t="s">
         <v>46</v>
@@ -8802,13 +8802,13 @@
         <v>1</v>
       </c>
       <c r="P12" s="16" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="Q12" s="16" t="s">
         <v>272</v>
       </c>
       <c r="R12" s="16" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="S12" s="16"/>
       <c r="T12" s="16"/>
@@ -8818,7 +8818,7 @@
         <v>178</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="C13" s="16" t="s">
         <v>283</v>
@@ -8836,7 +8836,7 @@
         <v>268</v>
       </c>
       <c r="H13" s="16" t="s">
-        <v>284</v>
+        <v>274</v>
       </c>
       <c r="I13" s="16" t="s">
         <v>46</v>
@@ -8854,13 +8854,13 @@
         <v>1</v>
       </c>
       <c r="P13" s="16" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="Q13" s="16" t="s">
         <v>272</v>
       </c>
       <c r="R13" s="16" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="S13" s="16"/>
       <c r="T13" s="16"/>
@@ -8870,7 +8870,7 @@
         <v>172</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C14" s="16" t="s">
         <v>283</v>
@@ -8888,7 +8888,7 @@
         <v>268</v>
       </c>
       <c r="H14" s="16" t="s">
-        <v>284</v>
+        <v>274</v>
       </c>
       <c r="I14" s="16" t="s">
         <v>46</v>
@@ -8906,13 +8906,13 @@
         <v>1</v>
       </c>
       <c r="P14" s="16" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="Q14" s="16" t="s">
         <v>272</v>
       </c>
       <c r="R14" s="16" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="S14" s="16"/>
       <c r="T14" s="16"/>
@@ -8922,7 +8922,7 @@
         <v>216</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C15" s="16" t="s">
         <v>89</v>
@@ -8966,7 +8966,7 @@
         <v>272</v>
       </c>
       <c r="R15" s="16" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="S15" s="16"/>
       <c r="T15" s="16"/>
@@ -8976,7 +8976,7 @@
         <v>245</v>
       </c>
       <c r="B16" s="16" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C16" s="16" t="s">
         <v>89</v>
@@ -9020,7 +9020,7 @@
         <v>272</v>
       </c>
       <c r="R16" s="16" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="S16" s="16"/>
       <c r="T16" s="16"/>
@@ -9030,7 +9030,7 @@
         <v>234</v>
       </c>
       <c r="B17" s="16" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="C17" s="16" t="s">
         <v>89</v>
@@ -9074,7 +9074,7 @@
         <v>272</v>
       </c>
       <c r="R17" s="16" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="S17" s="16"/>
       <c r="T17" s="16"/>
@@ -9084,7 +9084,7 @@
         <v>222</v>
       </c>
       <c r="B18" s="16" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C18" s="16" t="s">
         <v>89</v>
@@ -9128,7 +9128,7 @@
         <v>272</v>
       </c>
       <c r="R18" s="16" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="S18" s="16"/>
       <c r="T18" s="16"/>
@@ -9138,7 +9138,7 @@
         <v>239</v>
       </c>
       <c r="B19" s="16" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="C19" s="16" t="s">
         <v>89</v>
@@ -9182,7 +9182,7 @@
         <v>272</v>
       </c>
       <c r="R19" s="16" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="S19" s="16"/>
       <c r="T19" s="16"/>
@@ -9192,7 +9192,7 @@
         <v>97</v>
       </c>
       <c r="B20" s="16" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C20" s="16" t="s">
         <v>89</v>
@@ -9236,7 +9236,7 @@
         <v>272</v>
       </c>
       <c r="R20" s="16" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="S20" s="16"/>
       <c r="T20" s="16"/>
@@ -9246,7 +9246,7 @@
         <v>226</v>
       </c>
       <c r="B21" s="16" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C21" s="16" t="s">
         <v>89</v>
@@ -9290,7 +9290,7 @@
         <v>272</v>
       </c>
       <c r="R21" s="16" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="S21" s="16"/>
       <c r="T21" s="16"/>
@@ -9300,7 +9300,7 @@
         <v>105</v>
       </c>
       <c r="B22" s="16" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C22" s="16" t="s">
         <v>100</v>
@@ -9309,7 +9309,7 @@
         <v>99</v>
       </c>
       <c r="E22" s="16" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F22" s="9">
         <v>46155</v>
@@ -9318,7 +9318,7 @@
         <v>268</v>
       </c>
       <c r="H22" s="16" t="s">
-        <v>284</v>
+        <v>274</v>
       </c>
       <c r="I22" s="16" t="s">
         <v>46</v>
@@ -9346,17 +9346,17 @@
         <v>272</v>
       </c>
       <c r="R22" s="16" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="S22" s="16"/>
       <c r="T22" s="16"/>
     </row>
     <row r="23" spans="1:20" ht="18" customHeight="1">
       <c r="A23" s="16" t="s">
+        <v>297</v>
+      </c>
+      <c r="B23" s="16" t="s">
         <v>298</v>
-      </c>
-      <c r="B23" s="16" t="s">
-        <v>299</v>
       </c>
       <c r="C23" s="16" t="s">
         <v>100</v>
@@ -9374,7 +9374,7 @@
         <v>268</v>
       </c>
       <c r="H23" s="16" t="s">
-        <v>284</v>
+        <v>274</v>
       </c>
       <c r="I23" s="16" t="s">
         <v>46</v>
@@ -9402,7 +9402,7 @@
         <v>272</v>
       </c>
       <c r="R23" s="16" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="S23" s="16"/>
       <c r="T23" s="16"/>
@@ -9412,7 +9412,7 @@
         <v>110</v>
       </c>
       <c r="B24" s="16" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C24" s="16" t="s">
         <v>100</v>
@@ -9427,10 +9427,10 @@
         <v>46153</v>
       </c>
       <c r="G24" s="16" t="s">
+        <v>300</v>
+      </c>
+      <c r="H24" s="16" t="s">
         <v>301</v>
-      </c>
-      <c r="H24" s="16" t="s">
-        <v>302</v>
       </c>
       <c r="I24" s="16" t="s">
         <v>46</v>
@@ -9454,7 +9454,7 @@
         <v>272</v>
       </c>
       <c r="R24" s="16" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="S24" s="16"/>
       <c r="T24" s="16"/>
@@ -9464,7 +9464,7 @@
         <v>156</v>
       </c>
       <c r="B25" s="16" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C25" s="16" t="s">
         <v>100</v>
@@ -9482,7 +9482,7 @@
         <v>268</v>
       </c>
       <c r="H25" s="16" t="s">
-        <v>284</v>
+        <v>274</v>
       </c>
       <c r="I25" s="16" t="s">
         <v>46</v>
@@ -9496,7 +9496,7 @@
       <c r="L25" s="16"/>
       <c r="M25" s="16"/>
       <c r="N25" s="16" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="O25" s="16">
         <v>1</v>
@@ -9508,7 +9508,7 @@
         <v>272</v>
       </c>
       <c r="R25" s="16" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="S25" s="16"/>
       <c r="T25" s="16"/>
@@ -9518,7 +9518,7 @@
         <v>168</v>
       </c>
       <c r="B26" s="16" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C26" s="16" t="s">
         <v>100</v>
@@ -9536,7 +9536,7 @@
         <v>268</v>
       </c>
       <c r="H26" s="16" t="s">
-        <v>284</v>
+        <v>274</v>
       </c>
       <c r="I26" s="16" t="s">
         <v>46</v>
@@ -9560,7 +9560,7 @@
         <v>272</v>
       </c>
       <c r="R26" s="16" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="S26" s="16"/>
       <c r="T26" s="16"/>
@@ -9570,7 +9570,7 @@
         <v>160</v>
       </c>
       <c r="B27" s="16" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="C27" s="16" t="s">
         <v>100</v>
@@ -9588,7 +9588,7 @@
         <v>268</v>
       </c>
       <c r="H27" s="16" t="s">
-        <v>284</v>
+        <v>274</v>
       </c>
       <c r="I27" s="16" t="s">
         <v>46</v>
@@ -9602,7 +9602,7 @@
       <c r="L27" s="16"/>
       <c r="M27" s="16"/>
       <c r="N27" s="16" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="O27" s="16">
         <v>1</v>
@@ -9614,7 +9614,7 @@
         <v>272</v>
       </c>
       <c r="R27" s="16" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="S27" s="16"/>
       <c r="T27" s="16"/>
@@ -9624,7 +9624,7 @@
         <v>164</v>
       </c>
       <c r="B28" s="16" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C28" s="16" t="s">
         <v>100</v>
@@ -9642,7 +9642,7 @@
         <v>268</v>
       </c>
       <c r="H28" s="16" t="s">
-        <v>284</v>
+        <v>274</v>
       </c>
       <c r="I28" s="16" t="s">
         <v>46</v>
@@ -9656,7 +9656,7 @@
       <c r="L28" s="16"/>
       <c r="M28" s="16"/>
       <c r="N28" s="16" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="O28" s="16">
         <v>1</v>
@@ -9668,7 +9668,7 @@
         <v>272</v>
       </c>
       <c r="R28" s="16" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="S28" s="16"/>
       <c r="T28" s="16"/>
@@ -9678,7 +9678,7 @@
         <v>123</v>
       </c>
       <c r="B29" s="16" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="C29" s="16" t="s">
         <v>114</v>
@@ -9696,7 +9696,7 @@
         <v>268</v>
       </c>
       <c r="H29" s="16" t="s">
-        <v>284</v>
+        <v>274</v>
       </c>
       <c r="I29" s="16" t="s">
         <v>46</v>
@@ -9722,7 +9722,7 @@
         <v>272</v>
       </c>
       <c r="R29" s="16" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="S29" s="16"/>
       <c r="T29" s="16"/>
@@ -9732,7 +9732,7 @@
         <v>129</v>
       </c>
       <c r="B30" s="16" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C30" s="16" t="s">
         <v>114</v>
@@ -9776,7 +9776,7 @@
         <v>272</v>
       </c>
       <c r="R30" s="16" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="S30" s="16"/>
       <c r="T30" s="16"/>
@@ -9786,7 +9786,7 @@
         <v>141</v>
       </c>
       <c r="B31" s="16" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="C31" s="16" t="s">
         <v>114</v>
@@ -9830,7 +9830,7 @@
         <v>272</v>
       </c>
       <c r="R31" s="16" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="S31" s="16"/>
       <c r="T31" s="16"/>
@@ -9840,7 +9840,7 @@
         <v>137</v>
       </c>
       <c r="B32" s="16" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C32" s="16" t="s">
         <v>114</v>
@@ -9884,17 +9884,17 @@
         <v>272</v>
       </c>
       <c r="R32" s="16" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="S32" s="16"/>
       <c r="T32" s="16"/>
     </row>
     <row r="33" spans="1:20" ht="18" customHeight="1">
       <c r="A33" s="16" t="s">
+        <v>311</v>
+      </c>
+      <c r="B33" s="16" t="s">
         <v>312</v>
-      </c>
-      <c r="B33" s="16" t="s">
-        <v>313</v>
       </c>
       <c r="C33" s="16" t="s">
         <v>55</v>
@@ -9913,7 +9913,7 @@
         <v>269</v>
       </c>
       <c r="I33" s="16" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="J33" s="16" t="s">
         <v>270</v>
@@ -9936,7 +9936,7 @@
         <v>272</v>
       </c>
       <c r="R33" s="16" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="S33" s="16"/>
       <c r="T33" s="16"/>
@@ -9946,7 +9946,7 @@
         <v>146</v>
       </c>
       <c r="B34" s="16" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C34" s="16" t="s">
         <v>55</v>
@@ -9959,7 +9959,7 @@
         <v>46153</v>
       </c>
       <c r="G34" s="16" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="H34" s="16" t="s">
         <v>269</v>
@@ -9968,10 +9968,10 @@
         <v>46</v>
       </c>
       <c r="J34" s="16" t="s">
-        <v>273</v>
+        <v>316</v>
       </c>
       <c r="K34" s="16" t="s">
-        <v>273</v>
+        <v>316</v>
       </c>
       <c r="L34" s="16"/>
       <c r="M34" s="16"/>
@@ -9988,7 +9988,7 @@
         <v>272</v>
       </c>
       <c r="R34" s="16" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="S34" s="16"/>
       <c r="T34" s="16"/>
@@ -10014,7 +10014,7 @@
         <v>318</v>
       </c>
       <c r="H35" s="16" t="s">
-        <v>284</v>
+        <v>274</v>
       </c>
       <c r="I35" s="16" t="s">
         <v>62</v>
@@ -10040,7 +10040,7 @@
         <v>272</v>
       </c>
       <c r="R35" s="16" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="S35" s="16"/>
       <c r="T35" s="16"/>
@@ -10092,7 +10092,7 @@
         <v>272</v>
       </c>
       <c r="R36" s="16" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="S36" s="16"/>
       <c r="T36" s="16"/>
@@ -10719,7 +10719,7 @@
         <v>358</v>
       </c>
       <c r="B10" s="16">
-        <v>35</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -10727,7 +10727,7 @@
         <v>359</v>
       </c>
       <c r="B11" s="16">
-        <v>0</v>
+        <v>35</v>
       </c>
     </row>
     <row r="12" spans="1:2">

</xml_diff>

<commit_message>
Regenerate cached-run outputs and rebuild Anthony Le submission ZIP.
Reuse all 35 OpenAI cache entries with no fresh API extractions.
Keep presentation files out of the package. Relative source paths
and cached vs OpenAI-backed metrics are now in the workbooks and
run summary.

Co-authored-by: anthonyleedu <anthonyleedu@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/lisa_reconciliation.xlsx
+++ b/output/lisa_reconciliation.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1649" uniqueCount="399">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1653" uniqueCount="405">
   <si>
     <t>Priority</t>
   </si>
@@ -162,921 +162,927 @@
     <t>USD</t>
   </si>
   <si>
+    <t>data/confirmations/apex_02.pdf</t>
+  </si>
+  <si>
+    <t>APX-552544</t>
+  </si>
+  <si>
+    <t>ACTIVE</t>
+  </si>
+  <si>
+    <t>PO-4500050007</t>
+  </si>
+  <si>
+    <t>QTY_SHORT</t>
+  </si>
+  <si>
+    <t>Resolve 75-unit short confirmation on PO-4500050007 line 1 (BAR-A286-250) before release.</t>
+  </si>
+  <si>
+    <t>PROMISE_DATE</t>
+  </si>
+  <si>
+    <t>EXACT_CUSTOMER_PN</t>
+  </si>
+  <si>
+    <t>data/confirmations/apex_03.pdf</t>
+  </si>
+  <si>
+    <t>APX-978346</t>
+  </si>
+  <si>
+    <t>PO-4500050032</t>
+  </si>
+  <si>
+    <t>QuickShip Industrial</t>
+  </si>
+  <si>
+    <t>orders@quickship-ind.com</t>
+  </si>
+  <si>
+    <t>MISC-WAS-A25</t>
+  </si>
+  <si>
+    <t>Washer, A286, 0.25</t>
+  </si>
+  <si>
+    <t>NO_FORMAL_ACK_FOUND;INVOICE_NOT_ACK</t>
+  </si>
+  <si>
+    <t>No formal acknowledgment found for PO-4500050032 line 1. Request an order confirmation (the invoice/shipping notice is not sufficient).</t>
+  </si>
+  <si>
+    <t>data/confirmations/quickship_03.pdf</t>
+  </si>
+  <si>
+    <t>INFORMATIONAL</t>
+  </si>
+  <si>
+    <t>MISC-SPR-001</t>
+  </si>
+  <si>
+    <t>Spring, comp, 0.250 OD</t>
+  </si>
+  <si>
+    <t>No formal acknowledgment found for PO-4500050032 line 2. Request an order confirmation (the invoice/shipping notice is not sufficient).</t>
+  </si>
+  <si>
+    <t>PO-4500060619</t>
+  </si>
+  <si>
+    <t>APEX BAR &amp; TUBE CO.</t>
+  </si>
+  <si>
+    <t>UNKNOWN_PO</t>
+  </si>
+  <si>
+    <t>Verify whether this acknowledgment belongs to Beacon and whether PO number PO-4500060619 is correct.</t>
+  </si>
+  <si>
+    <t>data/confirmations/apex_rogue.pdf</t>
+  </si>
+  <si>
+    <t>APX-334543</t>
+  </si>
+  <si>
+    <t>PO-4500050002</t>
+  </si>
+  <si>
+    <t>BAR-CRES-250</t>
+  </si>
+  <si>
+    <t>CRES 17-4 PH bar stock, 0.250 dia</t>
+  </si>
+  <si>
+    <t>PRICE_HIGH</t>
+  </si>
+  <si>
+    <t>Confirm acceptance of $0.0902/unit increase (~2.30%) on PO-4500050002 line 1.</t>
+  </si>
+  <si>
+    <t>data/confirmations/apex_05.pdf</t>
+  </si>
+  <si>
+    <t>APX-389235</t>
+  </si>
+  <si>
+    <t>PO-4500050022</t>
+  </si>
+  <si>
+    <t>Continental Quality Heat Treat</t>
+  </si>
+  <si>
+    <t>info@continentalqht.com</t>
+  </si>
+  <si>
+    <t>HT-PRECIP</t>
+  </si>
+  <si>
+    <t>Precipitation heat treat A286, per lb</t>
+  </si>
+  <si>
+    <t>PRICE_NOT_STATED;PROMISE_LATE</t>
+  </si>
+  <si>
+    <t>Ask Continental Quality Heat Treat whether required date 2026-05-21 can be recovered; current promise is 21 days late.</t>
+  </si>
+  <si>
+    <t>SINGLE_REMAINING_LINE</t>
+  </si>
+  <si>
+    <t>data/confirmations/continental_01.pdf</t>
+  </si>
+  <si>
+    <t>PO-4500050012</t>
+  </si>
+  <si>
+    <t>Heritage Cold Heading</t>
+  </si>
+  <si>
+    <t>sales@heritagecoldheading.com</t>
+  </si>
+  <si>
+    <t>CHB-9472-4</t>
+  </si>
+  <si>
+    <t>APH-441-OS</t>
+  </si>
+  <si>
+    <t>Cold-headed blank for HX-9472-4</t>
+  </si>
+  <si>
+    <t>PROMISE_LATE</t>
+  </si>
+  <si>
+    <t>Ask Heritage Cold Heading whether required date 2026-06-04 can be recovered; current promise is 14 days late.</t>
+  </si>
+  <si>
+    <t>RULE_BASED</t>
+  </si>
+  <si>
+    <t>data/confirmations/heritage_06.pdf</t>
+  </si>
+  <si>
+    <t>HCH-74805</t>
+  </si>
+  <si>
+    <t>PO-4500050016</t>
+  </si>
+  <si>
+    <t>Liberty Surface Finishing</t>
+  </si>
+  <si>
+    <t>service@libertysurface.com</t>
+  </si>
+  <si>
+    <t>PLAT-PASV</t>
+  </si>
+  <si>
+    <t>Passivation per AMS 2700, per piece</t>
+  </si>
+  <si>
+    <t>Ask Liberty Surface Finishing whether required date 2026-05-17 can be recovered; current promise is 7 days late.</t>
+  </si>
+  <si>
+    <t>data/confirmations/liberty_01.pdf</t>
+  </si>
+  <si>
+    <t>LIB-PO-8573</t>
+  </si>
+  <si>
+    <t>PO-4500050019</t>
+  </si>
+  <si>
+    <t>PROMISE_MISSING</t>
+  </si>
+  <si>
+    <t>Request committed quantity and promise date for PO-4500050019 line 1 (PLAT-PASV).</t>
+  </si>
+  <si>
+    <t>data/confirmations/liberty_03.pdf</t>
+  </si>
+  <si>
+    <t>LIB-PO-9821</t>
+  </si>
+  <si>
+    <t>YELLOW</t>
+  </si>
+  <si>
+    <t>PO-4500050027</t>
+  </si>
+  <si>
+    <t>Ostmark Werkzeug GmbH</t>
+  </si>
+  <si>
+    <t>vertrieb@ostmark-wzg.de</t>
+  </si>
+  <si>
+    <t>TOOL-DIE-9472</t>
+  </si>
+  <si>
+    <t>Heading die set, 9472 profile</t>
+  </si>
+  <si>
+    <t>PROMISE_WINDOW_STRADDLES_REQUIRED</t>
+  </si>
+  <si>
+    <t>Delivery window for PO-4500050027 line 1 straddles required date 2026-05-15. Ask Ostmark Werkzeug GmbH to commit a date on or before 2026-05-15.</t>
+  </si>
+  <si>
+    <t>EUR</t>
+  </si>
+  <si>
+    <t>DELIVERY_WINDOW</t>
+  </si>
+  <si>
+    <t>EXACT_VENDOR_PN_TO_BEACON_PN</t>
+  </si>
+  <si>
+    <t>data/confirmations/ostmark_01.pdf</t>
+  </si>
+  <si>
+    <t>OST-220844</t>
+  </si>
+  <si>
+    <t>PO-4500050029</t>
+  </si>
+  <si>
+    <t>DATE_SEMANTICS_WARNING</t>
+  </si>
+  <si>
+    <t>Ostmark Werkzeug GmbH stated a ship date (not a Beacon receipt/promise date) on PO-4500050029. Confirm whether the ship date will still meet the required date at Beacon.</t>
+  </si>
+  <si>
+    <t>SHIP_DATE</t>
+  </si>
+  <si>
+    <t>data/confirmations/ostmark_02.pdf</t>
+  </si>
+  <si>
+    <t>OST-224427</t>
+  </si>
+  <si>
+    <t>TOOL-INS-CAR</t>
+  </si>
+  <si>
+    <t>OST-CAR-A-100</t>
+  </si>
+  <si>
+    <t>Carbide threading insert, A-series</t>
+  </si>
+  <si>
+    <t>Delivery window for PO-4500050027 line 2 straddles required date 2026-05-15. Ask Ostmark Werkzeug GmbH to commit a date on or before 2026-05-15.</t>
+  </si>
+  <si>
+    <t>PO-4500050028</t>
+  </si>
+  <si>
+    <t>Ostmark Werkzeug GmbH stated a ship date (not a Beacon receipt/promise date) on PO-4500050028. Confirm whether the ship date will still meet the required date at Beacon.</t>
+  </si>
+  <si>
+    <t>data/confirmations/ostmark_04.pdf</t>
+  </si>
+  <si>
+    <t>OST-226935</t>
+  </si>
+  <si>
+    <t>PO-4500050026</t>
+  </si>
+  <si>
+    <t>Ostmark Werkzeug GmbH stated a ship date (not a Beacon receipt/promise date) on PO-4500050026. Confirm whether the ship date will still meet the required date at Beacon.</t>
+  </si>
+  <si>
+    <t>data/confirmations/ostmark_03.pdf</t>
+  </si>
+  <si>
+    <t>OST-229377</t>
+  </si>
+  <si>
+    <t>PO-4500050030</t>
+  </si>
+  <si>
+    <t>DOCUMENT_REVISION;PRIOR_DOCUMENT_SUPERSEDED;DATE_SEMANTICS_WARNING</t>
+  </si>
+  <si>
+    <t>QuickShip Industrial stated a ship date (not a Beacon receipt/promise date) on PO-4500050030. Confirm whether the ship date will still meet the required date at Beacon.</t>
+  </si>
+  <si>
+    <t>data/confirmations/quickship_02.pdf</t>
+  </si>
+  <si>
+    <t>PO-4500050031</t>
+  </si>
+  <si>
+    <t>QuickShip Industrial stated a ship date (not a Beacon receipt/promise date) on PO-4500050031. Confirm whether the ship date will still meet the required date at Beacon.</t>
+  </si>
+  <si>
+    <t>data/confirmations/quickship_04.pdf</t>
+  </si>
+  <si>
+    <t>INFO</t>
+  </si>
+  <si>
+    <t>PO-4500050017</t>
+  </si>
+  <si>
+    <t>PLAT-CAD</t>
+  </si>
+  <si>
+    <t>Cadmium plating per QQ-P-416, per piece</t>
+  </si>
+  <si>
+    <t>PRICE_NOT_STATED</t>
+  </si>
+  <si>
+    <t>Confirmation for PO-4500050017 line 1 omits price; do not treat this as price acceptance.</t>
+  </si>
+  <si>
+    <t>data/confirmations/liberty_04.pdf</t>
+  </si>
+  <si>
+    <t>LIB-PO-9182</t>
+  </si>
+  <si>
+    <t>PO-4500050018</t>
+  </si>
+  <si>
+    <t>Confirmation for PO-4500050018 line 1 omits price; do not treat this as price acceptance.</t>
+  </si>
+  <si>
+    <t>data/confirmations/liberty_06.pdf</t>
+  </si>
+  <si>
+    <t>LIB-PO-9157</t>
+  </si>
+  <si>
+    <t>PO-4500050020</t>
+  </si>
+  <si>
+    <t>Confirmation for PO-4500050020 line 1 omits price; do not treat this as price acceptance.</t>
+  </si>
+  <si>
+    <t>data/confirmations/liberty_07.pdf</t>
+  </si>
+  <si>
+    <t>LIB-PO-9815</t>
+  </si>
+  <si>
+    <t>PO-4500050021</t>
+  </si>
+  <si>
+    <t>Confirmation for PO-4500050021 line 1 omits price; do not treat this as price acceptance.</t>
+  </si>
+  <si>
+    <t>data/confirmations/liberty_05.pdf</t>
+  </si>
+  <si>
+    <t>LIB-PO-9126</t>
+  </si>
+  <si>
+    <t>PO-4500050023</t>
+  </si>
+  <si>
+    <t>Confirmation for PO-4500050023 line 1 omits price; do not treat this as price acceptance.</t>
+  </si>
+  <si>
+    <t>data/confirmations/continental_04.pdf</t>
+  </si>
+  <si>
+    <t>CQH-42657</t>
+  </si>
+  <si>
+    <t>PO-4500050024</t>
+  </si>
+  <si>
+    <t>HT-SOLN</t>
+  </si>
+  <si>
+    <t>Solution treat + age, per lb</t>
+  </si>
+  <si>
+    <t>Confirmation for PO-4500050024 line 1 omits price; do not treat this as price acceptance.</t>
+  </si>
+  <si>
+    <t>data/confirmations/continental_03.pdf</t>
+  </si>
+  <si>
+    <t>CQH-40704</t>
+  </si>
+  <si>
+    <t>PO-4500050025</t>
+  </si>
+  <si>
+    <t>Confirmation for PO-4500050025 line 1 omits price; do not treat this as price acceptance.</t>
+  </si>
+  <si>
+    <t>data/confirmations/continental_02.pdf</t>
+  </si>
+  <si>
+    <t>GREEN</t>
+  </si>
+  <si>
+    <t>BAR-A286-375</t>
+  </si>
+  <si>
+    <t>A286 bar stock, 0.375 dia, mill-cert</t>
+  </si>
+  <si>
+    <t>Review PO-4500050001 line 1 with Apex Bar &amp; Tube Co..</t>
+  </si>
+  <si>
+    <t>PO-4500050003</t>
+  </si>
+  <si>
+    <t>Review PO-4500050003 line 1 with Apex Bar &amp; Tube Co..</t>
+  </si>
+  <si>
+    <t>data/confirmations/apex_07.pdf</t>
+  </si>
+  <si>
+    <t>APX-932684</t>
+  </si>
+  <si>
+    <t>PO-4500050004</t>
+  </si>
+  <si>
+    <t>Review PO-4500050004 line 1 with Apex Bar &amp; Tube Co..</t>
+  </si>
+  <si>
+    <t>data/confirmations/apex_01.pdf</t>
+  </si>
+  <si>
+    <t>APX-408970</t>
+  </si>
+  <si>
+    <t>PO-4500050005</t>
+  </si>
+  <si>
+    <t>Review PO-4500050005 line 1 with Apex Bar &amp; Tube Co..</t>
+  </si>
+  <si>
+    <t>data/confirmations/apex_08.pdf</t>
+  </si>
+  <si>
+    <t>APX-945201</t>
+  </si>
+  <si>
+    <t>PO-4500050006</t>
+  </si>
+  <si>
+    <t>Review PO-4500050006 line 1 with Apex Bar &amp; Tube Co..</t>
+  </si>
+  <si>
+    <t>data/confirmations/apex_06.pdf</t>
+  </si>
+  <si>
+    <t>APX-253836</t>
+  </si>
+  <si>
+    <t>PO-4500050008</t>
+  </si>
+  <si>
+    <t>Review PO-4500050008 line 1 with Apex Bar &amp; Tube Co..</t>
+  </si>
+  <si>
+    <t>data/confirmations/apex_04.pdf</t>
+  </si>
+  <si>
+    <t>APX-737955</t>
+  </si>
+  <si>
+    <t>BAR-TI64-188</t>
+  </si>
+  <si>
+    <t>Ti-6Al-4V bar stock, 0.188 dia</t>
+  </si>
+  <si>
+    <t>Review PO-4500050008 line 2 with Apex Bar &amp; Tube Co..</t>
+  </si>
+  <si>
+    <t>PO-4500050009</t>
+  </si>
+  <si>
+    <t>CHB-9472-3</t>
+  </si>
+  <si>
+    <t>APH-441</t>
+  </si>
+  <si>
+    <t>Cold-headed blank for HX-9472-3</t>
+  </si>
+  <si>
+    <t>Review PO-4500050009 line 1 with Heritage Cold Heading.</t>
+  </si>
+  <si>
+    <t>APPROVED_VENDOR_CROSSWALK</t>
+  </si>
+  <si>
+    <t>data/confirmations/heritage_01.pdf</t>
+  </si>
+  <si>
+    <t>HCH-75140</t>
+  </si>
+  <si>
+    <t>PO-4500050010</t>
+  </si>
+  <si>
+    <t>CHB-7715</t>
+  </si>
+  <si>
+    <t>Cold-headed blank for CSK-7715</t>
+  </si>
+  <si>
+    <t>Review PO-4500050010 line 1 with Heritage Cold Heading.</t>
+  </si>
+  <si>
+    <t>data/confirmations/heritage_04.pdf</t>
+  </si>
+  <si>
+    <t>HCH-77215</t>
+  </si>
+  <si>
+    <t>PO-4500050011</t>
+  </si>
+  <si>
+    <t>Review PO-4500050011 line 1 with Heritage Cold Heading.</t>
+  </si>
+  <si>
+    <t>data/confirmations/heritage_07.pdf</t>
+  </si>
+  <si>
+    <t>HCH-72939</t>
+  </si>
+  <si>
+    <t>CHB-3301</t>
+  </si>
+  <si>
+    <t>Cold-headed blank for NUT-3301-N</t>
+  </si>
+  <si>
+    <t>Review PO-4500050011 line 2 with Heritage Cold Heading.</t>
+  </si>
+  <si>
+    <t>Review PO-4500050011 line 3 with Heritage Cold Heading.</t>
+  </si>
+  <si>
+    <t>PO-4500050013</t>
+  </si>
+  <si>
+    <t>Review PO-4500050013 line 1 with Heritage Cold Heading.</t>
+  </si>
+  <si>
+    <t>data/confirmations/heritage_03.pdf</t>
+  </si>
+  <si>
+    <t>HCH-77346</t>
+  </si>
+  <si>
+    <t>Review PO-4500050013 line 2 with Heritage Cold Heading.</t>
+  </si>
+  <si>
+    <t>PO-4500050014</t>
+  </si>
+  <si>
+    <t>Review PO-4500050014 line 1 with Heritage Cold Heading.</t>
+  </si>
+  <si>
+    <t>data/confirmations/heritage_05.pdf</t>
+  </si>
+  <si>
+    <t>HCH-78781</t>
+  </si>
+  <si>
+    <t>Review PO-4500050014 line 2 with Heritage Cold Heading.</t>
+  </si>
+  <si>
+    <t>Review PO-4500050014 line 3 with Heritage Cold Heading.</t>
+  </si>
+  <si>
+    <t>PO-4500050015</t>
+  </si>
+  <si>
+    <t>Review PO-4500050015 line 1 with Heritage Cold Heading.</t>
+  </si>
+  <si>
+    <t>data/confirmations/heritage_02.pdf</t>
+  </si>
+  <si>
+    <t>HCH-75668</t>
+  </si>
+  <si>
+    <t>Review PO-4500050015 line 2 with Heritage Cold Heading.</t>
+  </si>
+  <si>
+    <t>Review PO-4500050015 line 3 with Heritage Cold Heading.</t>
+  </si>
+  <si>
+    <t>Source File</t>
+  </si>
+  <si>
+    <t>SHA256</t>
+  </si>
+  <si>
+    <t>Vendor (raw)</t>
+  </si>
+  <si>
+    <t>Document Number</t>
+  </si>
+  <si>
+    <t>Document Type</t>
+  </si>
+  <si>
+    <t>Commitment Status</t>
+  </si>
+  <si>
+    <t>Lifecycle</t>
+  </si>
+  <si>
+    <t>Revision?</t>
+  </si>
+  <si>
+    <t>Supersedes prior?</t>
+  </si>
+  <si>
+    <t>Part N</t>
+  </si>
+  <si>
+    <t>Part M</t>
+  </si>
+  <si>
+    <t>Currency</t>
+  </si>
+  <si>
+    <t>Line Count</t>
+  </si>
+  <si>
+    <t>Extraction Mode</t>
+  </si>
+  <si>
+    <t>Model</t>
+  </si>
+  <si>
+    <t>Cached?</t>
+  </si>
+  <si>
+    <t>Warnings</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>a2b124191abb</t>
+  </si>
+  <si>
+    <t>ACKNOWLEDGEMENT</t>
+  </si>
+  <si>
+    <t>FULL</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>NATIVE_TEXT</t>
+  </si>
+  <si>
+    <t>gpt-4o-mini</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>d41e5965ac0d</t>
+  </si>
+  <si>
+    <t>UNKNOWN</t>
+  </si>
+  <si>
+    <t>1e36a3bb8230</t>
+  </si>
+  <si>
+    <t>b109ebc6b485</t>
+  </si>
+  <si>
+    <t>527671baf80d</t>
+  </si>
+  <si>
+    <t>78e12caee3d0</t>
+  </si>
+  <si>
+    <t>3a93a05eccfb</t>
+  </si>
+  <si>
+    <t>498d9e57c248</t>
+  </si>
+  <si>
+    <t>666ddb95cb5e</t>
+  </si>
+  <si>
+    <t>171acbfe62b4</t>
+  </si>
+  <si>
+    <t>CONTINENTAL QUALITY HEAT TREAT</t>
+  </si>
+  <si>
+    <t>VISION</t>
+  </si>
+  <si>
+    <t>bccc160e1d7a</t>
+  </si>
+  <si>
+    <t>ce09a43a057d</t>
+  </si>
+  <si>
+    <t>0335b5f9c32c</t>
+  </si>
+  <si>
+    <t>955c6553efee</t>
+  </si>
+  <si>
+    <t>803cca7204dd</t>
+  </si>
+  <si>
+    <t>5c96fdc23f2b</t>
+  </si>
+  <si>
+    <t>da7824243c72</t>
+  </si>
+  <si>
+    <t>0f0f0358478e</t>
+  </si>
+  <si>
+    <t>33d82e21944f</t>
+  </si>
+  <si>
+    <t>22e8e11993b9</t>
+  </si>
+  <si>
+    <t>c4b891a575c5</t>
+  </si>
+  <si>
+    <t>LIB-PO-9240</t>
+  </si>
+  <si>
+    <t>data/confirmations/liberty_02.pdf</t>
+  </si>
+  <si>
+    <t>064f140583b6</t>
+  </si>
+  <si>
+    <t>df73e325ff79</t>
+  </si>
+  <si>
+    <t>RECEIPT_ONLY</t>
+  </si>
+  <si>
+    <t>RECEIPT_ACKNOWLEDGED_NO_SCHEDULE</t>
+  </si>
+  <si>
+    <t>e091bfef23ea</t>
+  </si>
+  <si>
+    <t>CAD</t>
+  </si>
+  <si>
+    <t>e8a55dd92b82</t>
+  </si>
+  <si>
+    <t>57987fd5631a</t>
+  </si>
+  <si>
+    <t>cb089f26bc54</t>
+  </si>
+  <si>
+    <t>7824420c3184</t>
+  </si>
+  <si>
+    <t>7dbe09998647</t>
+  </si>
+  <si>
+    <t>9e089392ebf2</t>
+  </si>
+  <si>
+    <t>af20c417f7de</t>
+  </si>
+  <si>
+    <t>data/confirmations/quickship_01.pdf</t>
+  </si>
+  <si>
+    <t>450c226ef559</t>
+  </si>
+  <si>
+    <t>SUPERSEDED</t>
+  </si>
+  <si>
+    <t>8c7d47657ef5</t>
+  </si>
+  <si>
+    <t>REVISION</t>
+  </si>
+  <si>
+    <t>e614ec5ee714</t>
+  </si>
+  <si>
+    <t>INVOICE</t>
+  </si>
+  <si>
+    <t>013b7d72a0f6</t>
+  </si>
+  <si>
+    <t>Vendor ID</t>
+  </si>
+  <si>
+    <t>Vendor Name</t>
+  </si>
+  <si>
+    <t>Vendor PN</t>
+  </si>
+  <si>
+    <t>Beacon PN</t>
+  </si>
+  <si>
+    <t>Evidence Count</t>
+  </si>
+  <si>
+    <t>Vendor PN Total</t>
+  </si>
+  <si>
+    <t>Purity</t>
+  </si>
+  <si>
+    <t>First Seen</t>
+  </si>
+  <si>
+    <t>Last Seen</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Source</t>
+  </si>
+  <si>
+    <t>V002</t>
+  </si>
+  <si>
+    <t>APH-125</t>
+  </si>
+  <si>
+    <t>APPROVED</t>
+  </si>
+  <si>
+    <t>historical_confirmation</t>
+  </si>
+  <si>
+    <t>APH-318</t>
+  </si>
+  <si>
+    <t>APH-4411</t>
+  </si>
+  <si>
+    <t>K-1050</t>
+  </si>
+  <si>
+    <t>CHB-5520</t>
+  </si>
+  <si>
+    <t>V005</t>
+  </si>
+  <si>
+    <t>TOOL-PUNCH-STD</t>
+  </si>
+  <si>
+    <t>WZ-9472-DS</t>
+  </si>
+  <si>
+    <t>WZ-HM-EIN</t>
+  </si>
+  <si>
+    <t>PROPOSED</t>
+  </si>
+  <si>
+    <t>current_document_context</t>
+  </si>
+  <si>
+    <t>Customer PN</t>
+  </si>
+  <si>
+    <t>Qty</t>
+  </si>
+  <si>
+    <t>Price</t>
+  </si>
+  <si>
+    <t>Explanation</t>
+  </si>
+  <si>
     <t>apex_02.pdf</t>
   </si>
   <si>
-    <t>APX-552544</t>
-  </si>
-  <si>
-    <t>ACTIVE</t>
-  </si>
-  <si>
-    <t>PO-4500050007</t>
-  </si>
-  <si>
-    <t>QTY_SHORT</t>
-  </si>
-  <si>
-    <t>Resolve 75-unit short confirmation on PO-4500050007 line 1 (BAR-A286-250) before release.</t>
-  </si>
-  <si>
-    <t>PROMISE_DATE</t>
-  </si>
-  <si>
-    <t>EXACT_CUSTOMER_PN</t>
-  </si>
-  <si>
-    <t>apex_03.pdf</t>
-  </si>
-  <si>
-    <t>APX-978346</t>
-  </si>
-  <si>
-    <t>PO-4500050032</t>
-  </si>
-  <si>
-    <t>QuickShip Industrial</t>
-  </si>
-  <si>
-    <t>orders@quickship-ind.com</t>
-  </si>
-  <si>
-    <t>MISC-WAS-A25</t>
-  </si>
-  <si>
-    <t>Washer, A286, 0.25</t>
-  </si>
-  <si>
-    <t>NO_FORMAL_ACK_FOUND;INVOICE_NOT_ACK</t>
-  </si>
-  <si>
-    <t>No formal acknowledgment found for PO-4500050032 line 1. Request an order confirmation (the invoice/shipping notice is not sufficient).</t>
-  </si>
-  <si>
-    <t>quickship_03.pdf</t>
-  </si>
-  <si>
-    <t>INFORMATIONAL</t>
-  </si>
-  <si>
-    <t>MISC-SPR-001</t>
-  </si>
-  <si>
-    <t>Spring, comp, 0.250 OD</t>
-  </si>
-  <si>
-    <t>No formal acknowledgment found for PO-4500050032 line 2. Request an order confirmation (the invoice/shipping notice is not sufficient).</t>
-  </si>
-  <si>
-    <t>PO-4500060619</t>
-  </si>
-  <si>
-    <t>APEX BAR &amp; TUBE CO.</t>
-  </si>
-  <si>
-    <t>UNKNOWN_PO</t>
-  </si>
-  <si>
-    <t>Verify whether this acknowledgment belongs to Beacon and whether PO number PO-4500060619 is correct.</t>
-  </si>
-  <si>
     <t>apex_rogue.pdf</t>
   </si>
   <si>
-    <t>APX-334543</t>
-  </si>
-  <si>
-    <t>PO-4500050002</t>
-  </si>
-  <si>
-    <t>BAR-CRES-250</t>
-  </si>
-  <si>
-    <t>CRES 17-4 PH bar stock, 0.250 dia</t>
-  </si>
-  <si>
-    <t>PRICE_HIGH</t>
-  </si>
-  <si>
-    <t>Confirm acceptance of $0.0902/unit increase (~2.30%) on PO-4500050002 line 1.</t>
-  </si>
-  <si>
-    <t>apex_05.pdf</t>
-  </si>
-  <si>
-    <t>APX-389235</t>
-  </si>
-  <si>
-    <t>PO-4500050022</t>
-  </si>
-  <si>
-    <t>Continental Quality Heat Treat</t>
-  </si>
-  <si>
-    <t>info@continentalqht.com</t>
-  </si>
-  <si>
-    <t>HT-PRECIP</t>
-  </si>
-  <si>
-    <t>Precipitation heat treat A286, per lb</t>
-  </si>
-  <si>
-    <t>PRICE_NOT_STATED;PROMISE_LATE</t>
-  </si>
-  <si>
-    <t>Ask Continental Quality Heat Treat whether required date 2026-05-21 can be recovered; current promise is 21 days late.</t>
-  </si>
-  <si>
-    <t>SINGLE_REMAINING_LINE</t>
-  </si>
-  <si>
-    <t>continental_01.pdf</t>
-  </si>
-  <si>
-    <t>PO-4500050012</t>
-  </si>
-  <si>
-    <t>Heritage Cold Heading</t>
-  </si>
-  <si>
-    <t>sales@heritagecoldheading.com</t>
-  </si>
-  <si>
-    <t>CHB-9472-4</t>
-  </si>
-  <si>
-    <t>APH-441-OS</t>
-  </si>
-  <si>
-    <t>Cold-headed blank for HX-9472-4</t>
-  </si>
-  <si>
-    <t>PROMISE_LATE</t>
-  </si>
-  <si>
-    <t>Ask Heritage Cold Heading whether required date 2026-06-04 can be recovered; current promise is 14 days late.</t>
-  </si>
-  <si>
-    <t>RULE_BASED</t>
-  </si>
-  <si>
-    <t>heritage_06.pdf</t>
-  </si>
-  <si>
-    <t>HCH-74805</t>
-  </si>
-  <si>
-    <t>PO-4500050016</t>
-  </si>
-  <si>
-    <t>Liberty Surface Finishing</t>
-  </si>
-  <si>
-    <t>service@libertysurface.com</t>
-  </si>
-  <si>
-    <t>PLAT-PASV</t>
-  </si>
-  <si>
-    <t>Passivation per AMS 2700, per piece</t>
-  </si>
-  <si>
-    <t>Ask Liberty Surface Finishing whether required date 2026-05-17 can be recovered; current promise is 7 days late.</t>
-  </si>
-  <si>
-    <t>liberty_01.pdf</t>
-  </si>
-  <si>
-    <t>LIB-PO-8573</t>
-  </si>
-  <si>
-    <t>PO-4500050019</t>
-  </si>
-  <si>
-    <t>PROMISE_MISSING</t>
-  </si>
-  <si>
-    <t>Request committed quantity and promise date for PO-4500050019 line 1 (PLAT-PASV).</t>
-  </si>
-  <si>
-    <t>liberty_03.pdf</t>
-  </si>
-  <si>
-    <t>LIB-PO-9821</t>
-  </si>
-  <si>
-    <t>YELLOW</t>
-  </si>
-  <si>
-    <t>PO-4500050027</t>
-  </si>
-  <si>
-    <t>Ostmark Werkzeug GmbH</t>
-  </si>
-  <si>
-    <t>vertrieb@ostmark-wzg.de</t>
-  </si>
-  <si>
-    <t>TOOL-DIE-9472</t>
-  </si>
-  <si>
-    <t>Heading die set, 9472 profile</t>
-  </si>
-  <si>
-    <t>PROMISE_WINDOW_STRADDLES_REQUIRED</t>
-  </si>
-  <si>
-    <t>Delivery window for PO-4500050027 line 1 straddles required date 2026-05-15. Ask Ostmark Werkzeug GmbH to commit a date on or before 2026-05-15.</t>
-  </si>
-  <si>
-    <t>EUR</t>
-  </si>
-  <si>
-    <t>DELIVERY_WINDOW</t>
-  </si>
-  <si>
-    <t>EXACT_VENDOR_PN_TO_BEACON_PN</t>
-  </si>
-  <si>
-    <t>ostmark_01.pdf</t>
-  </si>
-  <si>
-    <t>OST-220844</t>
-  </si>
-  <si>
-    <t>PO-4500050029</t>
-  </si>
-  <si>
-    <t>DATE_SEMANTICS_WARNING</t>
-  </si>
-  <si>
-    <t>Ostmark Werkzeug GmbH stated a ship date (not a Beacon receipt/promise date) on PO-4500050029. Confirm whether the ship date will still meet the required date at Beacon.</t>
-  </si>
-  <si>
-    <t>SHIP_DATE</t>
-  </si>
-  <si>
-    <t>ostmark_02.pdf</t>
-  </si>
-  <si>
-    <t>OST-224427</t>
-  </si>
-  <si>
-    <t>TOOL-INS-CAR</t>
-  </si>
-  <si>
-    <t>OST-CAR-A-100</t>
-  </si>
-  <si>
-    <t>Carbide threading insert, A-series</t>
-  </si>
-  <si>
-    <t>Delivery window for PO-4500050027 line 2 straddles required date 2026-05-15. Ask Ostmark Werkzeug GmbH to commit a date on or before 2026-05-15.</t>
-  </si>
-  <si>
-    <t>PO-4500050028</t>
-  </si>
-  <si>
-    <t>Ostmark Werkzeug GmbH stated a ship date (not a Beacon receipt/promise date) on PO-4500050028. Confirm whether the ship date will still meet the required date at Beacon.</t>
-  </si>
-  <si>
-    <t>ostmark_04.pdf</t>
-  </si>
-  <si>
-    <t>OST-226935</t>
-  </si>
-  <si>
-    <t>PO-4500050026</t>
-  </si>
-  <si>
-    <t>Ostmark Werkzeug GmbH stated a ship date (not a Beacon receipt/promise date) on PO-4500050026. Confirm whether the ship date will still meet the required date at Beacon.</t>
-  </si>
-  <si>
-    <t>ostmark_03.pdf</t>
-  </si>
-  <si>
-    <t>OST-229377</t>
-  </si>
-  <si>
-    <t>PO-4500050030</t>
-  </si>
-  <si>
-    <t>DOCUMENT_REVISION;PRIOR_DOCUMENT_SUPERSEDED;DATE_SEMANTICS_WARNING</t>
-  </si>
-  <si>
-    <t>QuickShip Industrial stated a ship date (not a Beacon receipt/promise date) on PO-4500050030. Confirm whether the ship date will still meet the required date at Beacon.</t>
-  </si>
-  <si>
-    <t>quickship_02.pdf</t>
-  </si>
-  <si>
-    <t>PO-4500050031</t>
-  </si>
-  <si>
-    <t>QuickShip Industrial stated a ship date (not a Beacon receipt/promise date) on PO-4500050031. Confirm whether the ship date will still meet the required date at Beacon.</t>
-  </si>
-  <si>
-    <t>quickship_04.pdf</t>
-  </si>
-  <si>
-    <t>INFO</t>
-  </si>
-  <si>
-    <t>PO-4500050017</t>
-  </si>
-  <si>
-    <t>PLAT-CAD</t>
-  </si>
-  <si>
-    <t>Cadmium plating per QQ-P-416, per piece</t>
-  </si>
-  <si>
-    <t>PRICE_NOT_STATED</t>
-  </si>
-  <si>
-    <t>Confirmation for PO-4500050017 line 1 omits price; do not treat this as price acceptance.</t>
-  </si>
-  <si>
-    <t>liberty_04.pdf</t>
-  </si>
-  <si>
-    <t>LIB-PO-9182</t>
-  </si>
-  <si>
-    <t>PO-4500050018</t>
-  </si>
-  <si>
-    <t>Confirmation for PO-4500050018 line 1 omits price; do not treat this as price acceptance.</t>
-  </si>
-  <si>
-    <t>liberty_06.pdf</t>
-  </si>
-  <si>
-    <t>LIB-PO-9157</t>
-  </si>
-  <si>
-    <t>PO-4500050020</t>
-  </si>
-  <si>
-    <t>Confirmation for PO-4500050020 line 1 omits price; do not treat this as price acceptance.</t>
-  </si>
-  <si>
-    <t>liberty_07.pdf</t>
-  </si>
-  <si>
-    <t>LIB-PO-9815</t>
-  </si>
-  <si>
-    <t>PO-4500050021</t>
-  </si>
-  <si>
-    <t>Confirmation for PO-4500050021 line 1 omits price; do not treat this as price acceptance.</t>
-  </si>
-  <si>
-    <t>liberty_05.pdf</t>
-  </si>
-  <si>
-    <t>LIB-PO-9126</t>
-  </si>
-  <si>
-    <t>PO-4500050023</t>
-  </si>
-  <si>
-    <t>Confirmation for PO-4500050023 line 1 omits price; do not treat this as price acceptance.</t>
-  </si>
-  <si>
-    <t>continental_04.pdf</t>
-  </si>
-  <si>
-    <t>CQH-42657</t>
-  </si>
-  <si>
-    <t>PO-4500050024</t>
-  </si>
-  <si>
-    <t>HT-SOLN</t>
-  </si>
-  <si>
-    <t>Solution treat + age, per lb</t>
-  </si>
-  <si>
-    <t>Confirmation for PO-4500050024 line 1 omits price; do not treat this as price acceptance.</t>
-  </si>
-  <si>
-    <t>continental_03.pdf</t>
-  </si>
-  <si>
-    <t>CQH-40704</t>
-  </si>
-  <si>
-    <t>PO-4500050025</t>
-  </si>
-  <si>
-    <t>Confirmation for PO-4500050025 line 1 omits price; do not treat this as price acceptance.</t>
-  </si>
-  <si>
-    <t>continental_02.pdf</t>
-  </si>
-  <si>
-    <t>GREEN</t>
-  </si>
-  <si>
-    <t>BAR-A286-375</t>
-  </si>
-  <si>
-    <t>A286 bar stock, 0.375 dia, mill-cert</t>
-  </si>
-  <si>
-    <t>Review PO-4500050001 line 1 with Apex Bar &amp; Tube Co..</t>
-  </si>
-  <si>
-    <t>PO-4500050003</t>
-  </si>
-  <si>
-    <t>Review PO-4500050003 line 1 with Apex Bar &amp; Tube Co..</t>
-  </si>
-  <si>
-    <t>apex_07.pdf</t>
-  </si>
-  <si>
-    <t>APX-932684</t>
-  </si>
-  <si>
-    <t>PO-4500050004</t>
-  </si>
-  <si>
-    <t>Review PO-4500050004 line 1 with Apex Bar &amp; Tube Co..</t>
-  </si>
-  <si>
-    <t>apex_01.pdf</t>
-  </si>
-  <si>
-    <t>APX-408970</t>
-  </si>
-  <si>
-    <t>PO-4500050005</t>
-  </si>
-  <si>
-    <t>Review PO-4500050005 line 1 with Apex Bar &amp; Tube Co..</t>
-  </si>
-  <si>
-    <t>apex_08.pdf</t>
-  </si>
-  <si>
-    <t>APX-945201</t>
-  </si>
-  <si>
-    <t>PO-4500050006</t>
-  </si>
-  <si>
-    <t>Review PO-4500050006 line 1 with Apex Bar &amp; Tube Co..</t>
-  </si>
-  <si>
-    <t>apex_06.pdf</t>
-  </si>
-  <si>
-    <t>APX-253836</t>
-  </si>
-  <si>
-    <t>PO-4500050008</t>
-  </si>
-  <si>
-    <t>Review PO-4500050008 line 1 with Apex Bar &amp; Tube Co..</t>
-  </si>
-  <si>
-    <t>apex_04.pdf</t>
-  </si>
-  <si>
-    <t>APX-737955</t>
-  </si>
-  <si>
-    <t>BAR-TI64-188</t>
-  </si>
-  <si>
-    <t>Ti-6Al-4V bar stock, 0.188 dia</t>
-  </si>
-  <si>
-    <t>Review PO-4500050008 line 2 with Apex Bar &amp; Tube Co..</t>
-  </si>
-  <si>
-    <t>PO-4500050009</t>
-  </si>
-  <si>
-    <t>CHB-9472-3</t>
-  </si>
-  <si>
-    <t>APH-441</t>
-  </si>
-  <si>
-    <t>Cold-headed blank for HX-9472-3</t>
-  </si>
-  <si>
-    <t>Review PO-4500050009 line 1 with Heritage Cold Heading.</t>
-  </si>
-  <si>
-    <t>APPROVED_VENDOR_CROSSWALK</t>
-  </si>
-  <si>
-    <t>heritage_01.pdf</t>
-  </si>
-  <si>
-    <t>HCH-75140</t>
-  </si>
-  <si>
-    <t>PO-4500050010</t>
-  </si>
-  <si>
-    <t>CHB-7715</t>
-  </si>
-  <si>
-    <t>Cold-headed blank for CSK-7715</t>
-  </si>
-  <si>
-    <t>Review PO-4500050010 line 1 with Heritage Cold Heading.</t>
-  </si>
-  <si>
-    <t>heritage_04.pdf</t>
-  </si>
-  <si>
-    <t>HCH-77215</t>
-  </si>
-  <si>
-    <t>PO-4500050011</t>
-  </si>
-  <si>
-    <t>Review PO-4500050011 line 1 with Heritage Cold Heading.</t>
-  </si>
-  <si>
-    <t>heritage_07.pdf</t>
-  </si>
-  <si>
-    <t>HCH-72939</t>
-  </si>
-  <si>
-    <t>CHB-3301</t>
-  </si>
-  <si>
-    <t>Cold-headed blank for NUT-3301-N</t>
-  </si>
-  <si>
-    <t>Review PO-4500050011 line 2 with Heritage Cold Heading.</t>
-  </si>
-  <si>
-    <t>Review PO-4500050011 line 3 with Heritage Cold Heading.</t>
-  </si>
-  <si>
-    <t>PO-4500050013</t>
-  </si>
-  <si>
-    <t>Review PO-4500050013 line 1 with Heritage Cold Heading.</t>
-  </si>
-  <si>
-    <t>heritage_03.pdf</t>
-  </si>
-  <si>
-    <t>HCH-77346</t>
-  </si>
-  <si>
-    <t>Review PO-4500050013 line 2 with Heritage Cold Heading.</t>
-  </si>
-  <si>
-    <t>PO-4500050014</t>
-  </si>
-  <si>
-    <t>Review PO-4500050014 line 1 with Heritage Cold Heading.</t>
-  </si>
-  <si>
-    <t>heritage_05.pdf</t>
-  </si>
-  <si>
-    <t>HCH-78781</t>
-  </si>
-  <si>
-    <t>Review PO-4500050014 line 2 with Heritage Cold Heading.</t>
-  </si>
-  <si>
-    <t>Review PO-4500050014 line 3 with Heritage Cold Heading.</t>
-  </si>
-  <si>
-    <t>PO-4500050015</t>
-  </si>
-  <si>
-    <t>Review PO-4500050015 line 1 with Heritage Cold Heading.</t>
-  </si>
-  <si>
-    <t>heritage_02.pdf</t>
-  </si>
-  <si>
-    <t>HCH-75668</t>
-  </si>
-  <si>
-    <t>Review PO-4500050015 line 2 with Heritage Cold Heading.</t>
-  </si>
-  <si>
-    <t>Review PO-4500050015 line 3 with Heritage Cold Heading.</t>
-  </si>
-  <si>
-    <t>Source File</t>
-  </si>
-  <si>
-    <t>SHA256</t>
-  </si>
-  <si>
-    <t>Vendor (raw)</t>
-  </si>
-  <si>
-    <t>Document Number</t>
-  </si>
-  <si>
-    <t>Document Type</t>
-  </si>
-  <si>
-    <t>Commitment Status</t>
-  </si>
-  <si>
-    <t>Lifecycle</t>
-  </si>
-  <si>
-    <t>Revision?</t>
-  </si>
-  <si>
-    <t>Supersedes prior?</t>
-  </si>
-  <si>
-    <t>Part N</t>
-  </si>
-  <si>
-    <t>Part M</t>
-  </si>
-  <si>
-    <t>Currency</t>
-  </si>
-  <si>
-    <t>Line Count</t>
-  </si>
-  <si>
-    <t>Extraction Mode</t>
-  </si>
-  <si>
-    <t>Model</t>
-  </si>
-  <si>
-    <t>Cached?</t>
-  </si>
-  <si>
-    <t>Warnings</t>
-  </si>
-  <si>
-    <t>Notes</t>
-  </si>
-  <si>
-    <t>a2b124191abb</t>
-  </si>
-  <si>
-    <t>ACKNOWLEDGEMENT</t>
-  </si>
-  <si>
-    <t>FULL</t>
-  </si>
-  <si>
-    <t>N</t>
-  </si>
-  <si>
-    <t>NATIVE_TEXT</t>
-  </si>
-  <si>
-    <t>gpt-4o-mini</t>
-  </si>
-  <si>
-    <t>Y</t>
-  </si>
-  <si>
-    <t>d41e5965ac0d</t>
-  </si>
-  <si>
-    <t>UNKNOWN</t>
-  </si>
-  <si>
-    <t>1e36a3bb8230</t>
-  </si>
-  <si>
-    <t>b109ebc6b485</t>
-  </si>
-  <si>
-    <t>527671baf80d</t>
-  </si>
-  <si>
-    <t>78e12caee3d0</t>
-  </si>
-  <si>
-    <t>3a93a05eccfb</t>
-  </si>
-  <si>
-    <t>498d9e57c248</t>
-  </si>
-  <si>
-    <t>666ddb95cb5e</t>
-  </si>
-  <si>
-    <t>171acbfe62b4</t>
-  </si>
-  <si>
-    <t>CONTINENTAL QUALITY HEAT TREAT</t>
-  </si>
-  <si>
-    <t>VISION</t>
-  </si>
-  <si>
-    <t>bccc160e1d7a</t>
-  </si>
-  <si>
-    <t>ce09a43a057d</t>
-  </si>
-  <si>
-    <t>0335b5f9c32c</t>
-  </si>
-  <si>
-    <t>955c6553efee</t>
-  </si>
-  <si>
-    <t>803cca7204dd</t>
-  </si>
-  <si>
-    <t>5c96fdc23f2b</t>
-  </si>
-  <si>
-    <t>da7824243c72</t>
-  </si>
-  <si>
-    <t>0f0f0358478e</t>
-  </si>
-  <si>
-    <t>33d82e21944f</t>
-  </si>
-  <si>
-    <t>22e8e11993b9</t>
-  </si>
-  <si>
-    <t>c4b891a575c5</t>
-  </si>
-  <si>
-    <t>LIB-PO-9240</t>
-  </si>
-  <si>
-    <t>liberty_02.pdf</t>
-  </si>
-  <si>
-    <t>064f140583b6</t>
-  </si>
-  <si>
-    <t>df73e325ff79</t>
-  </si>
-  <si>
-    <t>RECEIPT_ONLY</t>
-  </si>
-  <si>
-    <t>RECEIPT_ACKNOWLEDGED_NO_SCHEDULE</t>
-  </si>
-  <si>
-    <t>e091bfef23ea</t>
-  </si>
-  <si>
-    <t>CAD</t>
-  </si>
-  <si>
-    <t>e8a55dd92b82</t>
-  </si>
-  <si>
-    <t>57987fd5631a</t>
-  </si>
-  <si>
-    <t>cb089f26bc54</t>
-  </si>
-  <si>
-    <t>7824420c3184</t>
-  </si>
-  <si>
-    <t>7dbe09998647</t>
-  </si>
-  <si>
-    <t>9e089392ebf2</t>
-  </si>
-  <si>
-    <t>af20c417f7de</t>
-  </si>
-  <si>
-    <t>quickship_01.pdf</t>
-  </si>
-  <si>
-    <t>450c226ef559</t>
-  </si>
-  <si>
-    <t>SUPERSEDED</t>
-  </si>
-  <si>
-    <t>8c7d47657ef5</t>
-  </si>
-  <si>
-    <t>REVISION</t>
-  </si>
-  <si>
-    <t>e614ec5ee714</t>
-  </si>
-  <si>
-    <t>INVOICE</t>
-  </si>
-  <si>
-    <t>013b7d72a0f6</t>
-  </si>
-  <si>
-    <t>Vendor ID</t>
-  </si>
-  <si>
-    <t>Vendor Name</t>
-  </si>
-  <si>
-    <t>Vendor PN</t>
-  </si>
-  <si>
-    <t>Beacon PN</t>
-  </si>
-  <si>
-    <t>Evidence Count</t>
-  </si>
-  <si>
-    <t>Vendor PN Total</t>
-  </si>
-  <si>
-    <t>Purity</t>
-  </si>
-  <si>
-    <t>First Seen</t>
-  </si>
-  <si>
-    <t>Last Seen</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>Source</t>
-  </si>
-  <si>
-    <t>V002</t>
-  </si>
-  <si>
-    <t>APH-125</t>
-  </si>
-  <si>
-    <t>APPROVED</t>
-  </si>
-  <si>
-    <t>historical_confirmation</t>
-  </si>
-  <si>
-    <t>APH-318</t>
-  </si>
-  <si>
-    <t>APH-4411</t>
-  </si>
-  <si>
-    <t>K-1050</t>
-  </si>
-  <si>
-    <t>CHB-5520</t>
-  </si>
-  <si>
-    <t>V005</t>
-  </si>
-  <si>
-    <t>TOOL-PUNCH-STD</t>
-  </si>
-  <si>
-    <t>WZ-9472-DS</t>
-  </si>
-  <si>
-    <t>WZ-HM-EIN</t>
-  </si>
-  <si>
-    <t>PROPOSED</t>
-  </si>
-  <si>
-    <t>current_document_context</t>
-  </si>
-  <si>
-    <t>Customer PN</t>
-  </si>
-  <si>
-    <t>Qty</t>
-  </si>
-  <si>
-    <t>Price</t>
-  </si>
-  <si>
-    <t>Explanation</t>
-  </si>
-  <si>
     <t>Beacon Purchasing Copilot — Run Summary</t>
   </si>
   <si>
@@ -1104,13 +1110,22 @@
     <t>Scanned PDFs</t>
   </si>
   <si>
+    <t>OpenAI-backed documents</t>
+  </si>
+  <si>
+    <t>Native text + OpenAI (incl. cache)</t>
+  </si>
+  <si>
+    <t>Vision + OpenAI (incl. cache)</t>
+  </si>
+  <si>
+    <t>Fresh AI extractions this run</t>
+  </si>
+  <si>
     <t>Cached extractions</t>
   </si>
   <si>
-    <t>AI extractions</t>
-  </si>
-  <si>
-    <t>Local/OCR extractions</t>
+    <t>Local/OCR fallbacks</t>
   </si>
   <si>
     <t>Open PO lines</t>
@@ -1159,6 +1174,9 @@
   </si>
   <si>
     <t>QuickShip 'ship' dates are compared for visibility and flagged DATE_SEMANTICS_WARNING.</t>
+  </si>
+  <si>
+    <t>Cached OpenAI results still count as OpenAI-backed; Fresh AI extractions this run is the API-call count.</t>
   </si>
   <si>
     <t>Contact</t>
@@ -3629,26 +3647,6 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:AI19"/>
-  <hyperlinks>
-    <hyperlink ref="AF2" r:id="rId1"/>
-    <hyperlink ref="AF3" r:id="rId2"/>
-    <hyperlink ref="AF4" r:id="rId3"/>
-    <hyperlink ref="AF5" r:id="rId4"/>
-    <hyperlink ref="AF6" r:id="rId5"/>
-    <hyperlink ref="AF7" r:id="rId6"/>
-    <hyperlink ref="AF8" r:id="rId7"/>
-    <hyperlink ref="AF9" r:id="rId8"/>
-    <hyperlink ref="AF10" r:id="rId9"/>
-    <hyperlink ref="AF11" r:id="rId10"/>
-    <hyperlink ref="AF12" r:id="rId11"/>
-    <hyperlink ref="AF13" r:id="rId12"/>
-    <hyperlink ref="AF14" r:id="rId13"/>
-    <hyperlink ref="AF15" r:id="rId14"/>
-    <hyperlink ref="AF16" r:id="rId15"/>
-    <hyperlink ref="AF17" r:id="rId16"/>
-    <hyperlink ref="AF18" r:id="rId17"/>
-    <hyperlink ref="AF19" r:id="rId18"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -8090,53 +8088,6 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:AH46"/>
-  <hyperlinks>
-    <hyperlink ref="AE2" r:id="rId1"/>
-    <hyperlink ref="AE3" r:id="rId2"/>
-    <hyperlink ref="AE4" r:id="rId3"/>
-    <hyperlink ref="AE5" r:id="rId4"/>
-    <hyperlink ref="AE6" r:id="rId5"/>
-    <hyperlink ref="AE7" r:id="rId6"/>
-    <hyperlink ref="AE8" r:id="rId7"/>
-    <hyperlink ref="AE9" r:id="rId8"/>
-    <hyperlink ref="AE10" r:id="rId9"/>
-    <hyperlink ref="AE11" r:id="rId10"/>
-    <hyperlink ref="AE12" r:id="rId11"/>
-    <hyperlink ref="AE13" r:id="rId12"/>
-    <hyperlink ref="AE14" r:id="rId13"/>
-    <hyperlink ref="AE15" r:id="rId14"/>
-    <hyperlink ref="AE16" r:id="rId15"/>
-    <hyperlink ref="AE17" r:id="rId16"/>
-    <hyperlink ref="AE18" r:id="rId17"/>
-    <hyperlink ref="AE19" r:id="rId18"/>
-    <hyperlink ref="AE20" r:id="rId19"/>
-    <hyperlink ref="AE21" r:id="rId20"/>
-    <hyperlink ref="AE22" r:id="rId21"/>
-    <hyperlink ref="AE23" r:id="rId22"/>
-    <hyperlink ref="AE24" r:id="rId23"/>
-    <hyperlink ref="AE25" r:id="rId24"/>
-    <hyperlink ref="AE26" r:id="rId25"/>
-    <hyperlink ref="AE27" r:id="rId26"/>
-    <hyperlink ref="AE28" r:id="rId27"/>
-    <hyperlink ref="AE29" r:id="rId28"/>
-    <hyperlink ref="AE30" r:id="rId29"/>
-    <hyperlink ref="AE31" r:id="rId30"/>
-    <hyperlink ref="AE32" r:id="rId31"/>
-    <hyperlink ref="AE33" r:id="rId32"/>
-    <hyperlink ref="AE34" r:id="rId33"/>
-    <hyperlink ref="AE35" r:id="rId34"/>
-    <hyperlink ref="AE36" r:id="rId35"/>
-    <hyperlink ref="AE37" r:id="rId36"/>
-    <hyperlink ref="AE38" r:id="rId37"/>
-    <hyperlink ref="AE39" r:id="rId38"/>
-    <hyperlink ref="AE40" r:id="rId39"/>
-    <hyperlink ref="AE41" r:id="rId40"/>
-    <hyperlink ref="AE42" r:id="rId41"/>
-    <hyperlink ref="AE43" r:id="rId42"/>
-    <hyperlink ref="AE44" r:id="rId43"/>
-    <hyperlink ref="AE45" r:id="rId44"/>
-    <hyperlink ref="AE46" r:id="rId45"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -10100,43 +10051,6 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:T36"/>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1"/>
-    <hyperlink ref="A3" r:id="rId2"/>
-    <hyperlink ref="A4" r:id="rId3"/>
-    <hyperlink ref="A5" r:id="rId4"/>
-    <hyperlink ref="A6" r:id="rId5"/>
-    <hyperlink ref="A7" r:id="rId6"/>
-    <hyperlink ref="A8" r:id="rId7"/>
-    <hyperlink ref="A9" r:id="rId8"/>
-    <hyperlink ref="A10" r:id="rId9"/>
-    <hyperlink ref="A11" r:id="rId10"/>
-    <hyperlink ref="A12" r:id="rId11"/>
-    <hyperlink ref="A13" r:id="rId12"/>
-    <hyperlink ref="A14" r:id="rId13"/>
-    <hyperlink ref="A15" r:id="rId14"/>
-    <hyperlink ref="A16" r:id="rId15"/>
-    <hyperlink ref="A17" r:id="rId16"/>
-    <hyperlink ref="A18" r:id="rId17"/>
-    <hyperlink ref="A19" r:id="rId18"/>
-    <hyperlink ref="A20" r:id="rId19"/>
-    <hyperlink ref="A21" r:id="rId20"/>
-    <hyperlink ref="A22" r:id="rId21"/>
-    <hyperlink ref="A23" r:id="rId22"/>
-    <hyperlink ref="A24" r:id="rId23"/>
-    <hyperlink ref="A25" r:id="rId24"/>
-    <hyperlink ref="A26" r:id="rId25"/>
-    <hyperlink ref="A27" r:id="rId26"/>
-    <hyperlink ref="A28" r:id="rId27"/>
-    <hyperlink ref="A29" r:id="rId28"/>
-    <hyperlink ref="A30" r:id="rId29"/>
-    <hyperlink ref="A31" r:id="rId30"/>
-    <hyperlink ref="A32" r:id="rId31"/>
-    <hyperlink ref="A33" r:id="rId32"/>
-    <hyperlink ref="A34" r:id="rId33"/>
-    <hyperlink ref="A35" r:id="rId34"/>
-    <hyperlink ref="A36" r:id="rId35"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -10611,7 +10525,7 @@
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
       <c r="J2" s="4" t="s">
-        <v>44</v>
+        <v>349</v>
       </c>
       <c r="K2" s="4" t="s">
         <v>41</v>
@@ -10636,7 +10550,7 @@
       <c r="H3" s="4"/>
       <c r="I3" s="4"/>
       <c r="J3" s="4" t="s">
-        <v>70</v>
+        <v>350</v>
       </c>
       <c r="K3" s="4" t="s">
         <v>68</v>
@@ -10650,7 +10564,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B29"/>
+  <dimension ref="A1:B33"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="36.7109375" customWidth="1"/>
@@ -10659,25 +10573,25 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="17" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="18" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="19" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="B5" s="16">
         <v>35</v>
@@ -10685,7 +10599,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="19" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="B6" s="16">
         <v>32</v>
@@ -10693,7 +10607,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="19" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B7" s="16">
         <v>1</v>
@@ -10701,7 +10615,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="19" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="B8" s="16">
         <v>1</v>
@@ -10709,7 +10623,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="19" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="B9" s="16">
         <v>4</v>
@@ -10717,7 +10631,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="19" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B10" s="16">
         <v>35</v>
@@ -10725,63 +10639,63 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="19" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="B11" s="16">
-        <v>0</v>
+        <v>31</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="19" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="B12" s="16">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="19" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B13" s="16">
-        <v>44</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="19" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="B14" s="16">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="19" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B15" s="16">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="19" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="B16" s="16">
-        <v>10</v>
+        <v>44</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="19" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="B17" s="16">
-        <v>8</v>
+        <v>40</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="19" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="B18" s="16">
         <v>1</v>
@@ -10789,59 +10703,88 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="19" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="B19" s="16">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="19" t="s">
-        <v>368</v>
-      </c>
-      <c r="B20" s="16" t="s">
-        <v>369</v>
+        <v>370</v>
+      </c>
+      <c r="B20" s="16">
+        <v>8</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="19" t="s">
-        <v>370</v>
-      </c>
-      <c r="B21" s="16" t="s">
-        <v>272</v>
+        <v>371</v>
+      </c>
+      <c r="B21" s="16">
+        <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="19" t="s">
-        <v>371</v>
-      </c>
-      <c r="B22" s="16" t="s">
-        <v>270</v>
+        <v>372</v>
+      </c>
+      <c r="B22" s="16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2">
+      <c r="A23" s="19" t="s">
+        <v>373</v>
+      </c>
+      <c r="B23" s="16" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2">
+      <c r="A24" s="19" t="s">
+        <v>375</v>
+      </c>
+      <c r="B24" s="16" t="s">
+        <v>272</v>
       </c>
     </row>
     <row r="25" spans="1:2">
       <c r="A25" s="19" t="s">
-        <v>372</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2">
-      <c r="A26" s="18" t="s">
-        <v>373</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2">
-      <c r="A27" s="18" t="s">
-        <v>374</v>
+        <v>376</v>
+      </c>
+      <c r="B25" s="16" t="s">
+        <v>270</v>
       </c>
     </row>
     <row r="28" spans="1:2">
-      <c r="A28" s="18" t="s">
-        <v>375</v>
+      <c r="A28" s="19" t="s">
+        <v>377</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29" s="18" t="s">
-        <v>376</v>
+        <v>378</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2">
+      <c r="A30" s="18" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2">
+      <c r="A31" s="18" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2">
+      <c r="A32" s="18" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1">
+      <c r="A33" s="18" t="s">
+        <v>382</v>
       </c>
     </row>
   </sheetData>
@@ -10865,16 +10808,16 @@
         <v>4</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>377</v>
+        <v>383</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>378</v>
+        <v>384</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>379</v>
+        <v>385</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>380</v>
+        <v>386</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="80" customHeight="1">
@@ -10888,10 +10831,10 @@
         <v>36</v>
       </c>
       <c r="D2" s="16" t="s">
-        <v>381</v>
+        <v>387</v>
       </c>
       <c r="E2" s="16" t="s">
-        <v>382</v>
+        <v>388</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="80" customHeight="1">
@@ -10905,10 +10848,10 @@
         <v>47</v>
       </c>
       <c r="D3" s="16" t="s">
-        <v>383</v>
+        <v>389</v>
       </c>
       <c r="E3" s="16" t="s">
-        <v>384</v>
+        <v>390</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="80" customHeight="1">
@@ -10922,10 +10865,10 @@
         <v>54</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>385</v>
+        <v>391</v>
       </c>
       <c r="E4" s="16" t="s">
-        <v>386</v>
+        <v>392</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="80" customHeight="1">
@@ -10939,10 +10882,10 @@
         <v>66</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>387</v>
+        <v>393</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>388</v>
+        <v>394</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="80" customHeight="1">
@@ -10956,10 +10899,10 @@
         <v>72</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>389</v>
+        <v>395</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>390</v>
+        <v>396</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="80" customHeight="1">
@@ -10973,10 +10916,10 @@
         <v>79</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>391</v>
+        <v>397</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>392</v>
+        <v>398</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="80" customHeight="1">
@@ -10990,10 +10933,10 @@
         <v>88</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>393</v>
+        <v>399</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>394</v>
+        <v>400</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="80" customHeight="1">
@@ -11007,10 +10950,10 @@
         <v>99</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>395</v>
+        <v>401</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>396</v>
+        <v>402</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="80" customHeight="1">
@@ -11024,10 +10967,10 @@
         <v>107</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>397</v>
+        <v>403</v>
       </c>
       <c r="E10" s="16" t="s">
-        <v>398</v>
+        <v>404</v>
       </c>
     </row>
   </sheetData>

</xml_diff>